<commit_message>
Démo web avec événements fictifs, documentation des événements SKU
- Version web : page « Événements SKU » (onglets, filtres, détail, « Reprendre »),
  colonne « Événement », bandeau cliquable, garde-fou en 3 points avant le fichier LT et
  le zip de la Journée, fin des demandes boutique après export ; le moteur du navigateur
  reçoit les événements (mêmes quantités que l'outil installé, testé)
- Demande boutique fictive déplacée sur 7042.70 (ne croise plus l'allocation d'exemple)
- CLAUDE.md (patterns métier), README, décisions D-029 à D-033, questions Q-027 à Q-031

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jb2xnfp9PQKnevoHtuH3ZZ
</commit_message>
<xml_diff>
--- a/templates/evenements_sku.xlsx
+++ b/templates/evenements_sku.xlsx
@@ -808,12 +808,12 @@
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>La boutique demande du Melozio en plus (exemple fictif)</t>
+          <t>La boutique demande de l'Intenso en plus (exemple fictif)</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
-          <t>7005.70</t>
+          <t>7042.70</t>
         </is>
       </c>
       <c r="G5" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Événements SKU : allocation (vagues), quantité initiale de lancement et type Stock cible ; template unique (D-042)
Les allocations, lancements et stocks cibles saisis comme événements passent par le
même arbitrage métier qu'avant (calcul inchangé, parité 416/416). Une contradiction
entre deux sources bloque le SKU. Conversion des anciens fichiers : events_from_business.
Les modèles allocations.xlsx, launches.xlsx et target_stock.xlsx sont retirés.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BEvPQ8ejd6Ushnc12AaXPn
</commit_message>
<xml_diff>
--- a/templates/evenements_sku.xlsx
+++ b/templates/evenements_sku.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:T8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
@@ -867,6 +867,218 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Équipe</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Promotion</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Allocation AOS 14-21 oct</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Allocation officielle en deux vagues (exemple fictif)</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>7005.70</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>B80</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr"/>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>Allocation officielle (vagues)</t>
+        </is>
+      </c>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="inlineStr"/>
+      <c r="O6" s="1" t="inlineStr">
+        <is>
+          <t>Business (exemple)</t>
+        </is>
+      </c>
+      <c r="P6" s="1" t="inlineStr">
+        <is>
+          <t>Camille</t>
+        </is>
+      </c>
+      <c r="Q6" s="1" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="R6" s="1" t="inlineStr"/>
+      <c r="S6" s="1" t="inlineStr"/>
+      <c r="T6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Équipe</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Lancement</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Lancement Festive</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Quantité initiale avant le lancement (exemple fictif)</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>7200.70</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>B80</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr"/>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>Quantité initiale − Expected</t>
+        </is>
+      </c>
+      <c r="M7" s="1" t="n"/>
+      <c r="N7" s="1" t="inlineStr"/>
+      <c r="O7" s="1" t="inlineStr"/>
+      <c r="P7" s="1" t="inlineStr">
+        <is>
+          <t>Camille</t>
+        </is>
+      </c>
+      <c r="Q7" s="1" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="R7" s="1" t="inlineStr"/>
+      <c r="S7" s="1" t="inlineStr"/>
+      <c r="T7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>E7</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Équipe</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Stock cible</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Stock cible 142172</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Min / cible / max en boutique (exemple fictif)</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>142172</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>B80</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr"/>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr"/>
+      <c r="K8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>Min / cible / max</t>
+        </is>
+      </c>
+      <c r="M8" s="1" t="n"/>
+      <c r="N8" s="1" t="inlineStr"/>
+      <c r="O8" s="1" t="inlineStr"/>
+      <c r="P8" s="1" t="inlineStr">
+        <is>
+          <t>Camille</t>
+        </is>
+      </c>
+      <c r="Q8" s="1" t="inlineStr">
+        <is>
+          <t>Actif</t>
+        </is>
+      </c>
+      <c r="R8" s="1" t="inlineStr"/>
+      <c r="S8" s="1" t="inlineStr"/>
+      <c r="T8" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -878,13 +1090,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
     <col width="18" customWidth="1" style="1" min="2" max="2"/>
     <col width="18" customWidth="1" style="1" min="3" max="3"/>
     <col width="18" customWidth="1" style="1" min="4" max="4"/>
+    <col width="18" customWidth="1" style="1" min="5" max="5"/>
+    <col width="18" customWidth="1" style="1" min="6" max="6"/>
+    <col width="18" customWidth="1" style="1" min="7" max="7"/>
+    <col width="18" customWidth="1" style="1" min="8" max="8"/>
+    <col width="18" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -908,6 +1125,116 @@
           <t>Qty</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Déjà envoyé</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Vagues (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Vague en cours</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>E5</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>B80</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>7005.70</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>4800</v>
+      </c>
+      <c r="E2" s="1" t="inlineStr"/>
+      <c r="F2" s="1" t="inlineStr"/>
+      <c r="G2" s="1" t="inlineStr"/>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>75/25</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>E6</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>B80</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>7200.70</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr"/>
+      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr"/>
+      <c r="I3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>E7</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>B80</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>142172</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>30</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr"/>
+      <c r="I4" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -978,7 +1305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1352,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Promotion / Lancement / Arrêt d'envoi / Interdiction d'envoi / Conversion de SKU / Urgence / Demande boutique / À surveiller</t>
+          <t>Promotion / Lancement / Arrêt d'envoi / Interdiction d'envoi / Conversion de SKU / Urgence / Demande boutique / À surveiller / Stock cible</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1364,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Flag seulement / Quantité imposée / Quantité ajoutée / Bloquer l'envoi / Remplacer par un autre SKU</t>
+          <t>Flag seulement / Quantité imposée / Quantité ajoutée / Bloquer l'envoi / Remplacer par un autre SKU / Allocation officielle (vagues) / Quantité initiale − Expected / Min / cible / max</t>
         </is>
       </c>
     </row>
@@ -1116,46 +1443,82 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SKU détail</t>
+          <t>Allocation</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Facultatif : multiple d'un lancement absent de la Multiple list ; « Nouveau SKU » pour une conversion.</t>
+          <t>Type Promotion, effet « Allocation officielle (vagues) » : Qty = total, « Déjà envoyé », « Vagues (%) » (ex. 75/25, vide = une vague) et « Vague en cours » dans l'onglet « Quantités ». Fin vide permise. Remplace l'ancien allocations.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Demande boutique</t>
+          <t>Lancement</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Portée Personnel, une seule boutique ; « Demandé par » = prénom ou rôle, jamais d'email ; Échéance « Prochaine commande » ou vide.</t>
+          <t>Effet « Quantité initiale − Expected » : Qty = quantité initiale, Début = date de lancement. Remplace l'ancien launches.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ré-import</t>
+          <t>Stock cible</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Une Réf « #12 » met à jour l'événement n° 12 ; toute autre Réf en crée un.</t>
+          <t>Type Stock cible : Qty = cible, « Min » et « Max » obligatoires (onglet « Quantités »). Sous le min après commande → cible − Expected, arrondie au multiple ; au-dessus du max → plafonné. Remplace l'ancien target_stock.xlsx.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>SKU détail</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Facultatif : multiple d'un lancement absent de la Multiple list ; « Nouveau SKU » pour une conversion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Demande boutique</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Portée Personnel, une seule boutique ; « Demandé par » = prénom ou rôle, jamais d'email ; Échéance « Prochaine commande » ou vide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Ré-import</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Une Réf « #12 » met à jour l'événement n° 12 ; toute autre Réf en crée un.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Données</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Exemples fictifs. Ne jamais coller de contacts ni d'emails.</t>
         </is>

</xml_diff>

<commit_message>
Événements SKU : date de fin facultative pour tous les types, affichée « sans fin » (D-053)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BEvPQ8ejd6Ushnc12AaXPn
</commit_message>
<xml_diff>
--- a/templates/evenements_sku.xlsx
+++ b/templates/evenements_sku.xlsx
@@ -1424,7 +1424,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AAAA-MM-JJ ou JJ/MM/AAAA. Fin vide permise pour Arrêt et Interdiction.</t>
+          <t>AAAA-MM-JJ ou JJ/MM/AAAA. Début obligatoire ; Fin facultative (vide = sans fin, ex. une conversion effective à partir d'une date).</t>
         </is>
       </c>
     </row>
@@ -1448,7 +1448,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Type Promotion, effet « Allocation officielle (vagues) » : Qty = total, « Déjà envoyé », « Vagues (%) » (ex. 75/25, vide = une vague) et « Vague en cours » dans l'onglet « Quantités ». Fin vide permise. Remplace l'ancien allocations.xlsx.</t>
+          <t>Type Promotion, effet « Allocation officielle (vagues) » : Qty = total, « Déjà envoyé », « Vagues (%) » (ex. 75/25, vide = une vague) et « Vague en cours » dans l'onglet « Quantités ». Remplace l'ancien allocations.xlsx.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Événements SKU : statut calculé à partir des dates, arrêt manuel daté, dates « 22 oct. 2026 » (D-054)
Le statut affiché suit les dates (date du jour réelle) : À venir / Actif /
Terminé ; seuls Brouillon et Annulé restent manuels. « Terminer » met la fin
à aujourd'hui avec une trace dans l'historique, « Réactiver » l'efface. Les
anciens statuts « Terminé » sont relus comme un arrêt daté. Import Excel en
jour/mois/année (mois d'abord et année à 2 chiffres refusés). Démo web : même
règle, l'ancienne liste spc2_ev_done (cause du faux « Terminé ») est effacée.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BEvPQ8ejd6Ushnc12AaXPn
</commit_message>
<xml_diff>
--- a/templates/evenements_sku.xlsx
+++ b/templates/evenements_sku.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:T9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="1" min="1" max="1"/>
@@ -598,12 +598,12 @@
       <c r="H2" s="1" t="inlineStr"/>
       <c r="I2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>21/10/2026</t>
         </is>
       </c>
       <c r="K2" s="1" t="n">
@@ -632,7 +632,7 @@
       </c>
       <c r="Q2" s="1" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Selon les dates</t>
         </is>
       </c>
       <c r="R2" s="1" t="inlineStr"/>
@@ -678,12 +678,12 @@
       </c>
       <c r="I3" s="1" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
-          <t>2026-11-30</t>
+          <t>30/11/2026</t>
         </is>
       </c>
       <c r="K3" s="1" t="n">
@@ -710,7 +710,7 @@
       </c>
       <c r="Q3" s="1" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Selon les dates</t>
         </is>
       </c>
       <c r="R3" s="1" t="inlineStr"/>
@@ -756,7 +756,7 @@
       <c r="H4" s="1" t="inlineStr"/>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr"/>
@@ -778,7 +778,7 @@
       </c>
       <c r="Q4" s="1" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Selon les dates</t>
         </is>
       </c>
       <c r="R4" s="1" t="inlineStr"/>
@@ -824,7 +824,7 @@
       <c r="H5" s="1" t="inlineStr"/>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="J5" s="1" t="inlineStr"/>
@@ -848,7 +848,7 @@
       </c>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Selon les dates</t>
         </is>
       </c>
       <c r="R5" s="1" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="S5" s="1" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="T5" s="1" t="inlineStr">
@@ -906,7 +906,7 @@
       <c r="H6" s="1" t="inlineStr"/>
       <c r="I6" s="1" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="J6" s="1" t="inlineStr"/>
@@ -932,7 +932,7 @@
       </c>
       <c r="Q6" s="1" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Selon les dates</t>
         </is>
       </c>
       <c r="R6" s="1" t="inlineStr"/>
@@ -978,12 +978,12 @@
       <c r="H7" s="1" t="inlineStr"/>
       <c r="I7" s="1" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="J7" s="1" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>14/10/2026</t>
         </is>
       </c>
       <c r="K7" s="1" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="1" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Selon les dates</t>
         </is>
       </c>
       <c r="R7" s="1" t="inlineStr"/>
@@ -1050,7 +1050,7 @@
       <c r="H8" s="1" t="inlineStr"/>
       <c r="I8" s="1" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>05/10/2026</t>
         </is>
       </c>
       <c r="J8" s="1" t="inlineStr"/>
@@ -1072,12 +1072,88 @@
       </c>
       <c r="Q8" s="1" t="inlineStr">
         <is>
-          <t>Actif</t>
+          <t>Selon les dates</t>
         </is>
       </c>
       <c r="R8" s="1" t="inlineStr"/>
       <c r="S8" s="1" t="inlineStr"/>
       <c r="T8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>E8</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Équipe</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Promotion</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Free Gift (FG)</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Pochette offerte à l'achat (exemple fictif)</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>100924</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Toutes</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr"/>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>06/10/2026</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>22/10/2026</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1" t="inlineStr">
+        <is>
+          <t>Flag seulement</t>
+        </is>
+      </c>
+      <c r="M9" s="1" t="n"/>
+      <c r="N9" s="1" t="inlineStr"/>
+      <c r="O9" s="1" t="inlineStr">
+        <is>
+          <t>Marketing (exemple)</t>
+        </is>
+      </c>
+      <c r="P9" s="1" t="inlineStr">
+        <is>
+          <t>Camille</t>
+        </is>
+      </c>
+      <c r="Q9" s="1" t="inlineStr">
+        <is>
+          <t>Selon les dates</t>
+        </is>
+      </c>
+      <c r="R9" s="1" t="inlineStr"/>
+      <c r="S9" s="1" t="inlineStr"/>
+      <c r="T9" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1376,7 +1452,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Brouillon / Actif / Terminé / Annulé (vide = Actif)</t>
+          <t>Selon les dates (vide) / Brouillon / Annulé. À venir, actif ou terminé se calcule à partir des dates ; pour terminer, mets une date de fin.</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1500,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AAAA-MM-JJ ou JJ/MM/AAAA. Début obligatoire ; Fin facultative (vide = sans fin, ex. une conversion effective à partir d'une date).</t>
+          <t>Jour/mois/année : 22/10/2026 (ou une cellule date Excel). Début obligatoire ; Fin facultative (vide = sans fin, ex. une conversion effective à partir d'une date).</t>
         </is>
       </c>
     </row>

</xml_diff>